<commit_message>
## 代码重构第七期p4 - run_bech_suite优化
</commit_message>
<xml_diff>
--- a/docs_dev/审查日志与测试记录.xlsx
+++ b/docs_dev/审查日志与测试记录.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OpenProjects\RedstoneLink\rl-release-no-mixin\docs_dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E68CDF6-7A45-4E03-94FD-5B60E17E2806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE10F0E9-B11F-43A4-99DD-A3B25D11FBCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5136" yWindow="3816" windowWidth="23040" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="109">
   <si>
     <t>对象</t>
   </si>
@@ -427,6 +427,10 @@
   </si>
   <si>
     <t>代码重构p7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>t</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1675,6 +1679,9 @@
       <c r="A85" t="s">
         <v>107</v>
       </c>
+      <c r="C85" t="s">
+        <v>108</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>